<commit_message>
Update KiCad PCB, add build guide & backups
Apply multiple updates to the GoRAT project: modify the KiCad PCB (footprint/pad geometry, silkscreen labels, routing segments and UUIDs), and update accompanying KiCad project files and the GoRAT spreadsheet. Add Build_Guide.docx, LineDrawing PDFs and a technical SVG, and add new circuit diagram backup ZIPs dated 2026-03-24 while removing older March backup ZIPs. These edits refine silkscreen placement, pad shapes/sizes and routing for the current board revision.
</commit_message>
<xml_diff>
--- a/GORAT circuit diagram/GoRAT (version 1).xlsx
+++ b/GORAT circuit diagram/GoRAT (version 1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob-my.sharepoint.com/personal/nh22239_bristol_ac_uk/Documents/Documents/GitHub/GORAT-guitar-pedal/GORAT circuit diagram/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{67ECA503-9A80-4BD8-9DDB-9788C7FBB0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8FBB375-F8E5-42F3-A405-A7E059892484}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{67ECA503-9A80-4BD8-9DDB-9788C7FBB0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D688E8A6-60F0-4485-A700-95DFBB7E2F7B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8130C5E4-2DBF-402B-9F8C-66FE700F5F27}"/>
+    <workbookView xWindow="444" yWindow="0" windowWidth="22476" windowHeight="12336" xr2:uid="{8130C5E4-2DBF-402B-9F8C-66FE700F5F27}"/>
   </bookViews>
   <sheets>
     <sheet name="GoRAT (version 1)" sheetId="1" r:id="rId1"/>
@@ -1120,13 +1120,12 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="43"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -3002,7 +3001,7 @@
       <c r="D35">
         <v>1</v>
       </c>
-      <c r="E35" s="5">
+      <c r="E35">
         <f>5*Table1[[#This Row],[Qty]]</f>
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Update KiCad files: remap nets and rename caps
Synchronise PCB and schematic: remap many net indices across GORAT circuit diagram (.kicad_pcb, .kicad_sch, .kicad_prl, .kicad_pro) to match the schematic, and rename several capacitor references (e.g. C7/C15/C19 -> Cp7/Cp15/Cp19). Add autosave and CSV export files, update GoRAT spreadsheet, and refresh backup ZIPs (deleted older backups, added new ones). These changes ensure net and reference consistency between schematic and board files.
</commit_message>
<xml_diff>
--- a/GORAT circuit diagram/GoRAT (version 1).xlsx
+++ b/GORAT circuit diagram/GoRAT (version 1).xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob-my.sharepoint.com/personal/nh22239_bristol_ac_uk/Documents/Documents/GitHub/GORAT-guitar-pedal/GORAT circuit diagram/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{67ECA503-9A80-4BD8-9DDB-9788C7FBB0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D189E9CF-2D3B-458D-A095-ADDEF7E7F285}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{67ECA503-9A80-4BD8-9DDB-9788C7FBB0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C119F862-EFB3-4609-A5E5-28BD2724DB6C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8130C5E4-2DBF-402B-9F8C-66FE700F5F27}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{8130C5E4-2DBF-402B-9F8C-66FE700F5F27}"/>
   </bookViews>
   <sheets>
     <sheet name="GoRAT (version 1)" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1582,8 +1582,11 @@
     <col min="3" max="3" width="19.21875" customWidth="1"/>
     <col min="4" max="4" width="4.21875" customWidth="1"/>
     <col min="5" max="5" width="15.44140625" customWidth="1"/>
-    <col min="9" max="9" width="63.44140625" customWidth="1"/>
-    <col min="10" max="10" width="12.5546875" customWidth="1"/>
+    <col min="6" max="6" width="2.88671875" customWidth="1"/>
+    <col min="7" max="7" width="2.109375" customWidth="1"/>
+    <col min="8" max="8" width="2.88671875" customWidth="1"/>
+    <col min="9" max="9" width="20.77734375" customWidth="1"/>
+    <col min="10" max="10" width="8.5546875" customWidth="1"/>
     <col min="11" max="11" width="17.109375" customWidth="1"/>
     <col min="13" max="13" width="7.77734375" customWidth="1"/>
     <col min="14" max="14" width="19.44140625" customWidth="1"/>

</xml_diff>